<commit_message>
fix(sheets): dejar plantilla sin contestar para práctica estudiantil y pulir UX/UI del bloque de descarga
</commit_message>
<xml_diff>
--- a/public/descargas/practica-google-sheets-excel.xlsx
+++ b/public/descargas/practica-google-sheets-excel.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="109">
   <si>
     <t>MÓDULO 2: OFIMÁTICA EN LA NUBE</t>
   </si>
@@ -23,7 +23,7 @@
     <t>Práctica 1: Google Sheets / Microsoft Excel</t>
   </si>
   <si>
-    <t>Plantilla interactiva para laboratorio y autoestudio — Hojas de Cálculo</t>
+    <t>Cuaderno de práctica en blanco (Sin resolver) — Completa cada pestaña durante la clase</t>
   </si>
   <si>
     <t>Nombre del Alumno:</t>
@@ -35,79 +35,70 @@
     <t>Fecha:</t>
   </si>
   <si>
-    <t>29-08-2026</t>
-  </si>
-  <si>
     <t>Grupo / Grado:</t>
   </si>
   <si>
-    <t>📋 ESTRUCTURA DE LA PRÁCTICA (HOJAS DE TRABAJO)</t>
+    <t>📋 HOJAS DE TRABAJO A REALIZAR</t>
   </si>
   <si>
     <t>Pestaña 1: 1. Coordenadas y Tipos</t>
   </si>
   <si>
-    <t>Ubicación en el tablero y tipos de datos — Prueba Rápida 1 (C3, E7) y Prueba Rápida 2 (Texto vs Número vs Fórmula).</t>
-  </si>
-  <si>
-    <t>Por completar</t>
+    <t>Ubicación en el tablero y tipos de datos — Pruebas Rápidas 1 y 2: Ubicar celdas e identificar texto vs número vs fórmula.</t>
+  </si>
+  <si>
+    <t>[  ] Sin realizar</t>
   </si>
   <si>
     <t>Pestaña 2: 2. Fórmulas y Relleno</t>
   </si>
   <si>
-    <t>Signo igual (=) y autorrelleno inteligente — Prueba Rápida 3 (Multiplicación con celdas) y Prueba Rápida 4 (Series).</t>
+    <t>Signo igual (=) y autorrelleno inteligente — Pruebas Rápidas 3 y 4: Escribir fórmula con referencias y arrastrar series.</t>
   </si>
   <si>
     <t>Pestaña 3: 3. SUMA y PROMEDIO</t>
   </si>
   <si>
-    <t>Funciones con rangos (:) — Prueba Rápida 5 (Calificaciones con =SUMA() y =PROMEDIO()).</t>
+    <t>Funciones con rangos (:) — Prueba Rápida 5: Escribir las funciones =SUMA() y =PROMEDIO().</t>
   </si>
   <si>
     <t>Pestaña 4: 4. Cotización Gamer</t>
   </si>
   <si>
-    <t>Proyecto Integrador de Laboratorio — Cotización completa con subtotales, total general, promedio y formato $.</t>
-  </si>
-  <si>
-    <t>💡 INSTRUCCIONES PARA EL ESTUDIANTE:</t>
-  </si>
-  <si>
-    <t>1. Navega entre las pestañas usando las pestañas inferiores de la ventana.</t>
-  </si>
-  <si>
-    <t>2. Las celdas con fondo AMARILLO son tus espacios de trabajo donde debes escribir o ingresar fórmulas.</t>
-  </si>
-  <si>
-    <t>3. Recuerda que toda fórmula SIEMPRE comienza con el signo igual (=).</t>
-  </si>
-  <si>
-    <t>4. Al finalizar todas las hojas, guarda tu archivo como "Presupuesto_TuNombre.xlsx" y entrégalo.</t>
+    <t>Proyecto Integrador de Laboratorio — Calcular subtotales con fórmula, total general, promedio y aplicar formato $.</t>
+  </si>
+  <si>
+    <t>💡 INSTRUCCIONES PARA RESOLVER TU PRÁCTICA:</t>
+  </si>
+  <si>
+    <t>1. Este archivo es tu plantilla de trabajo. Todas las actividades vienen SIN RESOLVER para que tú practiques.</t>
+  </si>
+  <si>
+    <t>2. Las celdas marcadas en color AMARILLO son tus espacios de trabajo: allí debes escribir tus datos o tus fórmulas.</t>
+  </si>
+  <si>
+    <t>3. Recuerda: Toda fórmula SIEMPRE comienza con el signo igual (=).</t>
+  </si>
+  <si>
+    <t>4. Al terminar todos los ejercicios, guarda el archivo como "Presupuesto_TuNombre.xlsx" para entregarlo.</t>
   </si>
   <si>
     <t>ACTIVIDAD 1 &amp; 2: COORDENADAS Y TIPOS DE DATOS</t>
   </si>
   <si>
-    <t>[Escribe tu nombre aquí]</t>
-  </si>
-  <si>
     <t>🎯 PRUEBA RÁPIDA 1: Ubicación en el Tablero de Coordenadas</t>
   </si>
   <si>
-    <t>Paso 1: Haz clic en la celda C3 y escribe tu nombre.</t>
-  </si>
-  <si>
-    <t>Paso 2: Haz clic en la celda E7 y escribe tu comida favorita.</t>
-  </si>
-  <si>
-    <t>[Escribe tu comida favorita]</t>
-  </si>
-  <si>
-    <t>🎯 PRUEBA RÁPIDA 2: Identificación de Tipos de Datos</t>
-  </si>
-  <si>
-    <t>Escribe exactamente el dato indicado en las celdas amarillas y observa su alineación automática:</t>
+    <t>1. Haz clic en la celda C3 (fondo amarillo) y escribe tu nombre completo.</t>
+  </si>
+  <si>
+    <t>2. Haz clic en la celda E7 (fondo amarillo) y escribe el nombre de tu comida favorita.</t>
+  </si>
+  <si>
+    <t>🎯 PRUEBA RÁPIDA 2: Identificación de Tipos de Datos (Texto vs Número)</t>
+  </si>
+  <si>
+    <t>Escribe exactamente el texto/número en la celda amarilla y luego anota hacia dónde se alineó automáticamente:</t>
   </si>
   <si>
     <t>Ubicación</t>
@@ -119,10 +110,10 @@
     <t>Escríbelo Aquí</t>
   </si>
   <si>
-    <t>Tipo de Dato</t>
-  </si>
-  <si>
-    <t>Alineación Obtenida</t>
+    <t>¿Qué Tipo de Dato es?</t>
+  </si>
+  <si>
+    <t>Alineación Observada</t>
   </si>
   <si>
     <t>Celda D13</t>
@@ -131,37 +122,22 @@
     <t>Audífonos</t>
   </si>
   <si>
-    <t>Texto</t>
-  </si>
-  <si>
-    <t>Izquierda</t>
-  </si>
-  <si>
     <t>Celda D14</t>
   </si>
   <si>
     <t>350</t>
   </si>
   <si>
-    <t>Número</t>
-  </si>
-  <si>
-    <t>Derecha</t>
-  </si>
-  <si>
     <t>Celda D15</t>
   </si>
   <si>
     <t>350 pesos</t>
   </si>
   <si>
-    <t>❓ PREGUNTA DE COMPROBACIÓN:</t>
-  </si>
-  <si>
-    <t>¿Por qué en la celda con "350 pesos" la hoja clasifica el dato como Texto e impide hacer sumas?</t>
-  </si>
-  <si>
-    <t>[ Tu respuesta: Al incluir letras (pesos), la hoja no reconoce el valor como un número puro. Para mostrar el signo de pesos sin convertirlo en texto, se debe aplicar Formato de Moneda ($) ]</t>
+    <t>❓ PREGUNTA DE REFLEXIÓN:</t>
+  </si>
+  <si>
+    <t>¿Por qué en la celda con "350 pesos" la hoja no permite realizar cálculos matemáticos?</t>
   </si>
   <si>
     <t>ACTIVIDAD 3 &amp; 4: FÓRMULAS CON REFERENCIAS Y AUTORRELLENO</t>
@@ -191,7 +167,7 @@
     <t>Precio Unitario (C7)</t>
   </si>
   <si>
-    <t>Valor inicial ($50)</t>
+    <t>Valor inicial</t>
   </si>
   <si>
     <t>Enero</t>
@@ -200,21 +176,21 @@
     <t>Cantidad (C8)</t>
   </si>
   <si>
-    <t>Cantidad de piezas (3)</t>
+    <t>Cantidad fija</t>
   </si>
   <si>
     <t>Subtotal (C9)</t>
   </si>
   <si>
-    <t>Escribe =C7*C8</t>
-  </si>
-  <si>
-    <t>🧪 Reto de comprobación en clase:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Cambia el Precio en C7 de 50 a 120.
-2. Presiona Enter.
-3. Comprueba que C9 se actualiza automáticamente a 360.</t>
+    <t>Escribe aquí la fórmula =C7*C8</t>
+  </si>
+  <si>
+    <t>🧪 Reto de comprobación:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Escribe la fórmula =C7*C8 en C9 y presiona Enter.
+2. Ahora cambia el Precio en C7 de 50 a 120.
+3. Observa cómo el resultado se actualiza automáticamente a 360.</t>
   </si>
   <si>
     <t xml:space="preserve">Instrucciones:
@@ -228,7 +204,7 @@
     <t>🎯 PRUEBA RÁPIDA 5: Cálculo de Calificaciones</t>
   </si>
   <si>
-    <t>Ingresa las fórmulas con las funciones =SUMA() y =PROMEDIO() en las celdas amarillas:</t>
+    <t>Escribe las fórmulas con las funciones =SUMA() y =PROMEDIO() en las celdas amarillas:</t>
   </si>
   <si>
     <t>Evaluación / Parcial</t>
@@ -237,68 +213,68 @@
     <t>Calificación</t>
   </si>
   <si>
-    <t>Fórmula Requerida</t>
-  </si>
-  <si>
-    <t>Significado del Rango ( : )</t>
+    <t>Tu Fórmula a Escribir</t>
+  </si>
+  <si>
+    <t>Instrucción / Rango a Usar</t>
   </si>
   <si>
     <t>Parcial 1</t>
   </si>
   <si>
-    <t>Dato numérico</t>
-  </si>
-  <si>
-    <t>Celda C8</t>
+    <t>Dato</t>
+  </si>
+  <si>
+    <t>Celda individual C8</t>
   </si>
   <si>
     <t>Parcial 2</t>
   </si>
   <si>
-    <t>Celda C9</t>
+    <t>Celda individual C9</t>
   </si>
   <si>
     <t>Parcial 3</t>
   </si>
   <si>
-    <t>Celda C10</t>
+    <t>Celda individual C10</t>
   </si>
   <si>
     <t>Parcial 4</t>
   </si>
   <si>
-    <t>Celda C11</t>
+    <t>Celda individual C11</t>
   </si>
   <si>
     <t>TOTAL PUNTOS</t>
   </si>
   <si>
-    <t>=SUMA(C8:C11)</t>
-  </si>
-  <si>
-    <t>Suma el bloque continuo desde C8 hasta C11.</t>
+    <t>Escribe aquí: =SUMA(C8:C11)</t>
+  </si>
+  <si>
+    <t>Usa la función SUMA sobre el rango continuo C8:C11.</t>
   </si>
   <si>
     <t>PROMEDIO FINAL</t>
   </si>
   <si>
-    <t>=PROMEDIO(C8:C11)</t>
-  </si>
-  <si>
-    <t>Calcula la media aritmética del rango.</t>
+    <t>Escribe aquí: =PROMEDIO(C8:C11)</t>
+  </si>
+  <si>
+    <t>Calcula la media aritmética de las 4 calificaciones.</t>
   </si>
   <si>
     <t>💡 RECORDATORIO SOBRE RANGOS:</t>
   </si>
   <si>
-    <t xml:space="preserve">Los dos puntos ( : ) indican "hasta". La expresión C8:C11 incluye: C8, C9, C10 y C11.
-Si usas punto y coma o coma (C8, C11), solo se tomarían dos celdas sueltas.</t>
+    <t xml:space="preserve">Los dos puntos ( : ) indican "desde... hasta". La expresión C8:C11 toma todas las celdas desde C8 hasta C11.
+Si usaras una coma (C8, C11), solo tomaría esas dos celdas sueltas.</t>
   </si>
   <si>
     <t>PROYECTO DE LABORATORIO: COTIZACIÓN TIENDA GAMER</t>
   </si>
   <si>
-    <t>Calcula subtotales con fórmulas, total con SUMA, promedio con PROMEDIO y aplica formato $.</t>
+    <t>Reto: Calcula todos los subtotales con fórmula, el total general con SUMA y el precio promedio con PROMEDIO.</t>
   </si>
   <si>
     <t>Producto</t>
@@ -307,25 +283,25 @@
     <t>Cantidad</t>
   </si>
   <si>
-    <t>Precio Unitario ($)</t>
-  </si>
-  <si>
-    <t>Subtotal ($)</t>
-  </si>
-  <si>
-    <t>📝 GUÍA DE PASOS:</t>
+    <t>Precio Unitario</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>📝 INSTRUCCIONES PASO A PASO:</t>
   </si>
   <si>
     <t>Teclado Mecánico RGB</t>
   </si>
   <si>
-    <t>Paso 1: En E6 escribe =C6*D6.</t>
+    <t>Paso 1: En la celda E6 escribe la fórmula =C6*D6.</t>
   </si>
   <si>
     <t>Mouse Inalámbrico</t>
   </si>
   <si>
-    <t>Paso 2: Arrastra el cuadro azul hasta E10 para copiar la fórmula.</t>
+    <t>Paso 2: Arrastra el cuadro azul desde E6 hasta E10 para copiar la fórmula a todos los productos.</t>
   </si>
   <si>
     <t>Monitor 144Hz</t>
@@ -343,7 +319,7 @@
     <t>Headset con Micrófono</t>
   </si>
   <si>
-    <t>Paso 5: Aplica formato de Moneda ($) con Ctrl + Shift + 4.</t>
+    <t>Paso 5: Selecciona precios y subtotales y aplica formato de Moneda ($).</t>
   </si>
   <si>
     <t>TOTAL GENERAL</t>
@@ -355,7 +331,7 @@
     <t>✅ LISTA DE COTEJO Y AUTOEVALUACIÓN:</t>
   </si>
   <si>
-    <t xml:space="preserve"> [   ] Subtotales calculados con coordenadas de celda (=C6*D6)</t>
+    <t xml:space="preserve"> [   ] Subtotales calculados con fórmula de multiplicación (=C6*D6)</t>
   </si>
   <si>
     <t xml:space="preserve"> [   ] Fórmula copiada correctamente en toda la columna con el controlador de relleno</t>
@@ -380,7 +356,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -444,25 +420,46 @@
     </font>
     <font>
       <b/>
-      <color rgb="0284C7"/>
+      <color rgb="FFFFFF"/>
       <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F172A"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="D97706"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="64748B"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
       <color rgb="7C3AED"/>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFF"/>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
+      <sz val="13"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -472,47 +469,15 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
       <b/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="D97706"/>
+      <color rgb="0F172A"/>
       <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="64748B"/>
-      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
       <b/>
       <color rgb="059669"/>
       <sz val="11"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="0F172A"/>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="7C3AED"/>
-      <sz val="13"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -536,22 +501,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="E0F2FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="0F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F1F5F9"/>
+        <fgColor rgb="F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -584,6 +549,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="EAB308"/>
+      </left>
+      <right style="medium">
+        <color rgb="EAB308"/>
+      </right>
+      <top style="medium">
+        <color rgb="EAB308"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="EAB308"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="CBD5E1"/>
       </left>
@@ -598,135 +578,113 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="1E293B"/>
-      </left>
-      <right style="medium">
-        <color rgb="1E293B"/>
-      </right>
-      <top style="medium">
-        <color rgb="1E293B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="1E293B"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1115,10 +1073,10 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>7</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>4</v>
@@ -1126,7 +1084,7 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -1134,55 +1092,55 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>9</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>10</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>12</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>13</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>15</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>16</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>17</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
@@ -1190,7 +1148,7 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -1198,7 +1156,7 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
@@ -1206,7 +1164,7 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
@@ -1214,7 +1172,7 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
@@ -1248,15 +1206,16 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="4" width="24" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -1264,131 +1223,131 @@
       <c r="F2" s="13"/>
     </row>
     <row r="3" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="15" t="s">
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+    </row>
+    <row r="7" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E7" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-    </row>
-    <row r="7" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="17" t="s">
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="16" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
+      <c r="D12" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="E12" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="F12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="18" t="s">
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="C13" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="D13" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="17" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="D14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E13" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>45</v>
-      </c>
       <c r="D15" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="11" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
@@ -1396,29 +1355,29 @@
       <c r="F18" s="11"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
+      <c r="B19" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
+      <c r="B20" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1453,7 +1412,7 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="13" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -1462,115 +1421,115 @@
       <c r="G2" s="13"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="F4" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="14"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="24">
         <v>50</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="F4" s="15" t="s">
+      <c r="D7" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="G4" s="15"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="22" t="s">
+      <c r="G7" s="27">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C8" s="24">
+        <v>3</v>
+      </c>
+      <c r="D8" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="F8" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="C9" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="G6" s="23" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="25">
-        <v>50</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" s="28">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="25">
-        <v>3</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G8" s="28">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="29">
-        <f>C7*C8</f>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G9" s="24" t="s">
+      <c r="F9" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" s="28" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F10" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" s="24" t="s">
+      <c r="F10" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" s="28" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="31" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C11" s="31"/>
       <c r="D11" s="31"/>
-      <c r="F11" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G11" s="24" t="s">
+      <c r="F11" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" s="28" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="32" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C12" s="32"/>
       <c r="D12" s="32"/>
-      <c r="F12" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="24" t="s">
+      <c r="F12" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="28" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1584,7 +1543,7 @@
       <c r="C14" s="32"/>
       <c r="D14" s="32"/>
       <c r="F14" s="33" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="G14" s="33"/>
     </row>
@@ -1624,129 +1583,129 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" s="13" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
       <c r="E2" s="13"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
+      <c r="B4" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
+      <c r="B5" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E7" s="34" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="24" t="s">
-        <v>74</v>
+      <c r="B8" s="23" t="s">
+        <v>66</v>
       </c>
       <c r="C8" s="35">
         <v>8</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" s="36" t="s">
-        <v>76</v>
+        <v>67</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
-        <v>77</v>
+      <c r="B9" s="23" t="s">
+        <v>69</v>
       </c>
       <c r="C9" s="35">
         <v>9</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="36" t="s">
-        <v>78</v>
+        <v>67</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="24" t="s">
-        <v>79</v>
+      <c r="B10" s="23" t="s">
+        <v>71</v>
       </c>
       <c r="C10" s="35">
         <v>10</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>80</v>
+        <v>67</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="24" t="s">
-        <v>81</v>
+      <c r="B11" s="23" t="s">
+        <v>73</v>
       </c>
       <c r="C11" s="35">
         <v>7</v>
       </c>
       <c r="D11" s="36" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="36" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="37" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" s="38">
-        <f>SUM(C8:C11)</f>
-      </c>
-      <c r="D12" s="39" t="s">
-        <v>84</v>
+      <c r="C12" s="39" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>76</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="41">
-        <f>AVERAGE(C8:C11)</f>
-      </c>
-      <c r="D13" s="39" t="s">
-        <v>87</v>
+      <c r="B13" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>79</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -1754,7 +1713,7 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -1788,168 +1747,168 @@
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="42" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="43" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="44" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="17">
+        <v>2</v>
+      </c>
+      <c r="D6" s="45">
+        <v>850</v>
+      </c>
+      <c r="E6" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="43" t="s">
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="44" t="s">
+      <c r="C7" s="17">
+        <v>3</v>
+      </c>
+      <c r="D7" s="45">
+        <v>450</v>
+      </c>
+      <c r="E7" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="44" t="s">
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="C8" s="17">
+        <v>1</v>
+      </c>
+      <c r="D8" s="45">
+        <v>3200</v>
+      </c>
+      <c r="E8" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="E5" s="44" t="s">
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="C9" s="17">
+        <v>4</v>
+      </c>
+      <c r="D9" s="45">
+        <v>200</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="47" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="24" t="s">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C10" s="17">
         <v>2</v>
       </c>
-      <c r="D6" s="46">
-        <v>850</v>
-      </c>
-      <c r="E6" s="47">
-        <f>C6*D6</f>
-      </c>
-      <c r="F6" s="48" t="s">
+      <c r="D10" s="45">
+        <v>950</v>
+      </c>
+      <c r="E10" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="47" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="19">
-        <v>3</v>
-      </c>
-      <c r="D7" s="46">
-        <v>450</v>
-      </c>
-      <c r="E7" s="47">
-        <f>C7*D7</f>
-      </c>
-      <c r="F7" s="48" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="C8" s="19">
-        <v>1</v>
-      </c>
-      <c r="D8" s="46">
-        <v>3200</v>
-      </c>
-      <c r="E8" s="47">
-        <f>C8*D8</f>
-      </c>
-      <c r="F8" s="48" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="19">
-        <v>4</v>
-      </c>
-      <c r="D9" s="46">
-        <v>200</v>
-      </c>
-      <c r="E9" s="47">
-        <f>C9*D9</f>
-      </c>
-      <c r="F9" s="48" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="19">
-        <v>2</v>
-      </c>
-      <c r="D10" s="46">
-        <v>950</v>
-      </c>
-      <c r="E10" s="47">
-        <f>C10*D10</f>
-      </c>
-      <c r="F10" s="48" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="49" t="s">
-        <v>108</v>
-      </c>
-      <c r="C11" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="E11" s="51">
-        <f>SUM(E6:E10)</f>
+        <v>100</v>
+      </c>
+      <c r="C11" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="53">
-        <f>AVERAGE(D6:D10)</f>
-      </c>
-      <c r="E12" s="50" t="s">
+      <c r="B12" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="28" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="54" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
+      <c r="B15" s="51" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -1958,7 +1917,7 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
@@ -1967,7 +1926,7 @@
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
@@ -1976,7 +1935,7 @@
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
@@ -1985,7 +1944,7 @@
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
@@ -1994,7 +1953,7 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>

</xml_diff>